<commit_message>
cleaned and rebased data, polishing left....
</commit_message>
<xml_diff>
--- a/clean data/clean.xlsx
+++ b/clean data/clean.xlsx
@@ -1091,7 +1091,7 @@
         <v>45261</v>
       </c>
       <c r="C23" t="n">
-        <v>124345.9</v>
+        <v>62173</v>
       </c>
       <c r="D23" t="n">
         <v>185.7</v>
@@ -1120,7 +1120,7 @@
         <v>45231</v>
       </c>
       <c r="C24" t="n">
-        <v>121571.9</v>
+        <v>60786.12</v>
       </c>
       <c r="D24" t="n">
         <v>186.3</v>
@@ -1149,7 +1149,7 @@
         <v>45200</v>
       </c>
       <c r="C25" t="n">
-        <v>117546.4</v>
+        <v>58773</v>
       </c>
       <c r="D25" t="n">
         <v>185.3</v>
@@ -1178,7 +1178,7 @@
         <v>45170</v>
       </c>
       <c r="C26" t="n">
-        <v>117485</v>
+        <v>58743.45</v>
       </c>
       <c r="D26" t="n">
         <v>184.1</v>
@@ -1207,7 +1207,7 @@
         <v>45139</v>
       </c>
       <c r="C27" t="n">
-        <v>117475.9</v>
+        <v>58738.31</v>
       </c>
       <c r="D27" t="n">
         <v>186.2</v>
@@ -1236,7 +1236,7 @@
         <v>45108</v>
       </c>
       <c r="C28" t="n">
-        <v>117843.42</v>
+        <v>58922.09</v>
       </c>
       <c r="D28" t="n">
         <v>186.3</v>
@@ -1265,7 +1265,7 @@
         <v>45078</v>
       </c>
       <c r="C29" t="n">
-        <v>118112.76</v>
+        <v>59056.12</v>
       </c>
       <c r="D29" t="n">
         <v>181</v>
@@ -1294,7 +1294,7 @@
         <v>45047</v>
       </c>
       <c r="C30" t="n">
-        <v>121165.54</v>
+        <v>60583</v>
       </c>
       <c r="D30" t="n">
         <v>179.1</v>
@@ -1323,7 +1323,7 @@
         <v>45017</v>
       </c>
       <c r="C31" t="n">
-        <v>120290.48</v>
+        <v>60145.25</v>
       </c>
       <c r="D31" t="n">
         <v>178.1</v>
@@ -1352,7 +1352,7 @@
         <v>44986</v>
       </c>
       <c r="C32" t="n">
-        <v>115027.34</v>
+        <v>57514</v>
       </c>
       <c r="D32" t="n">
         <v>177.2</v>
@@ -1381,7 +1381,7 @@
         <v>44958</v>
       </c>
       <c r="C33" t="n">
-        <v>113291.2</v>
+        <v>56646</v>
       </c>
       <c r="D33" t="n">
         <v>176.8</v>
@@ -1410,7 +1410,7 @@
         <v>44927</v>
       </c>
       <c r="C34" t="n">
-        <v>112492.66</v>
+        <v>56246.1</v>
       </c>
       <c r="D34" t="n">
         <v>176.5</v>

</xml_diff>